<commit_message>
walk through the pooled pathway and profile steps
</commit_message>
<xml_diff>
--- a/04_Continuous_no_group/03_Profile_Clusters/c_data/profile_clusters.xlsx
+++ b/04_Continuous_no_group/03_Profile_Clusters/c_data/profile_clusters.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6718" uniqueCount="4387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6733" uniqueCount="4396">
   <si>
     <t>sheet</t>
   </si>
@@ -12662,6 +12662,12 @@
     <t>1.32.0</t>
   </si>
   <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
+  </si>
+  <si>
     <t>farver</t>
   </si>
   <si>
@@ -12875,6 +12881,12 @@
     <t>1.52.0</t>
   </si>
   <si>
+    <t>knitr</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
     <t>labeling</t>
   </si>
   <si>
@@ -12896,9 +12908,6 @@
     <t>lifecycle</t>
   </si>
   <si>
-    <t>1.0.5</t>
-  </si>
-  <si>
     <t>magrittr</t>
   </si>
   <si>
@@ -13046,6 +13055,12 @@
     <t>rlang</t>
   </si>
   <si>
+    <t>rmarkdown</t>
+  </si>
+  <si>
+    <t>2.31</t>
+  </si>
+  <si>
     <t>rprojroot</t>
   </si>
   <si>
@@ -13148,6 +13163,12 @@
     <t>tzdb</t>
   </si>
   <si>
+    <t>utf8</t>
+  </si>
+  <si>
+    <t>1.2.6</t>
+  </si>
+  <si>
     <t>vctrs</t>
   </si>
   <si>
@@ -13164,6 +13185,12 @@
   </si>
   <si>
     <t>3.0.2</t>
+  </si>
+  <si>
+    <t>xfun</t>
+  </si>
+  <si>
+    <t>0.57</t>
   </si>
   <si>
     <t>XVector</t>
@@ -60259,7 +60286,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -60652,7 +60679,7 @@
         <v>4221</v>
       </c>
       <c r="B36" t="s">
-        <v>4210</v>
+        <v>4222</v>
       </c>
       <c r="C36" t="s">
         <v>4155</v>
@@ -60660,10 +60687,10 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>4222</v>
+        <v>4223</v>
       </c>
       <c r="B37" t="s">
-        <v>4223</v>
+        <v>4210</v>
       </c>
       <c r="C37" t="s">
         <v>4155</v>
@@ -60729,21 +60756,21 @@
         <v>4234</v>
       </c>
       <c r="B43" t="s">
-        <v>4210</v>
+        <v>4235</v>
       </c>
       <c r="C43" t="s">
-        <v>4163</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>4235</v>
+        <v>4236</v>
       </c>
       <c r="B44" t="s">
-        <v>4236</v>
+        <v>4210</v>
       </c>
       <c r="C44" t="s">
-        <v>4155</v>
+        <v>4163</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -60809,7 +60836,7 @@
         <v>4248</v>
       </c>
       <c r="C50" t="s">
-        <v>4158</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -60817,18 +60844,18 @@
         <v>4249</v>
       </c>
       <c r="B51" t="s">
-        <v>4229</v>
+        <v>4250</v>
       </c>
       <c r="C51" t="s">
-        <v>4155</v>
+        <v>4158</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>4250</v>
+        <v>4251</v>
       </c>
       <c r="B52" t="s">
-        <v>4251</v>
+        <v>4231</v>
       </c>
       <c r="C52" t="s">
         <v>4155</v>
@@ -60842,29 +60869,29 @@
         <v>4253</v>
       </c>
       <c r="C53" t="s">
-        <v>4254</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
+        <v>4254</v>
+      </c>
+      <c r="B54" t="s">
         <v>4255</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>4256</v>
-      </c>
-      <c r="C54" t="s">
-        <v>4257</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
+        <v>4257</v>
+      </c>
+      <c r="B55" t="s">
         <v>4258</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
         <v>4259</v>
-      </c>
-      <c r="C55" t="s">
-        <v>4155</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -60872,21 +60899,21 @@
         <v>4260</v>
       </c>
       <c r="B56" t="s">
-        <v>4210</v>
+        <v>4261</v>
       </c>
       <c r="C56" t="s">
-        <v>4163</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>4261</v>
+        <v>4262</v>
       </c>
       <c r="B57" t="s">
-        <v>4262</v>
+        <v>4210</v>
       </c>
       <c r="C57" t="s">
-        <v>4155</v>
+        <v>4163</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -60949,18 +60976,18 @@
         <v>4273</v>
       </c>
       <c r="B63" t="s">
-        <v>4177</v>
+        <v>4274</v>
       </c>
       <c r="C63" t="s">
-        <v>4163</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>4274</v>
+        <v>4275</v>
       </c>
       <c r="B64" t="s">
-        <v>4275</v>
+        <v>4177</v>
       </c>
       <c r="C64" t="s">
         <v>4163</v>
@@ -60974,7 +61001,7 @@
         <v>4277</v>
       </c>
       <c r="C65" t="s">
-        <v>4158</v>
+        <v>4163</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -60985,7 +61012,7 @@
         <v>4279</v>
       </c>
       <c r="C66" t="s">
-        <v>4155</v>
+        <v>4158</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -61007,7 +61034,7 @@
         <v>4283</v>
       </c>
       <c r="C68" t="s">
-        <v>4158</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -61018,7 +61045,7 @@
         <v>4285</v>
       </c>
       <c r="C69" t="s">
-        <v>4155</v>
+        <v>4158</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -61070,7 +61097,7 @@
         <v>4294</v>
       </c>
       <c r="B74" t="s">
-        <v>4295</v>
+        <v>4214</v>
       </c>
       <c r="C74" t="s">
         <v>4155</v>
@@ -61078,10 +61105,10 @@
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
+        <v>4295</v>
+      </c>
+      <c r="B75" t="s">
         <v>4296</v>
-      </c>
-      <c r="B75" t="s">
-        <v>4297</v>
       </c>
       <c r="C75" t="s">
         <v>4155</v>
@@ -61089,10 +61116,10 @@
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
+        <v>4297</v>
+      </c>
+      <c r="B76" t="s">
         <v>4298</v>
-      </c>
-      <c r="B76" t="s">
-        <v>4299</v>
       </c>
       <c r="C76" t="s">
         <v>4155</v>
@@ -61100,10 +61127,10 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
+        <v>4299</v>
+      </c>
+      <c r="B77" t="s">
         <v>4300</v>
-      </c>
-      <c r="B77" t="s">
-        <v>4301</v>
       </c>
       <c r="C77" t="s">
         <v>4155</v>
@@ -61111,10 +61138,10 @@
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
+        <v>4301</v>
+      </c>
+      <c r="B78" t="s">
         <v>4302</v>
-      </c>
-      <c r="B78" t="s">
-        <v>4303</v>
       </c>
       <c r="C78" t="s">
         <v>4155</v>
@@ -61122,10 +61149,10 @@
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
+        <v>4303</v>
+      </c>
+      <c r="B79" t="s">
         <v>4304</v>
-      </c>
-      <c r="B79" t="s">
-        <v>4305</v>
       </c>
       <c r="C79" t="s">
         <v>4155</v>
@@ -61133,10 +61160,10 @@
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
+        <v>4305</v>
+      </c>
+      <c r="B80" t="s">
         <v>4306</v>
-      </c>
-      <c r="B80" t="s">
-        <v>4307</v>
       </c>
       <c r="C80" t="s">
         <v>4155</v>
@@ -61144,10 +61171,10 @@
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
+        <v>4307</v>
+      </c>
+      <c r="B81" t="s">
         <v>4308</v>
-      </c>
-      <c r="B81" t="s">
-        <v>4309</v>
       </c>
       <c r="C81" t="s">
         <v>4155</v>
@@ -61155,10 +61182,10 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
+        <v>4309</v>
+      </c>
+      <c r="B82" t="s">
         <v>4310</v>
-      </c>
-      <c r="B82" t="s">
-        <v>4311</v>
       </c>
       <c r="C82" t="s">
         <v>4155</v>
@@ -61166,10 +61193,10 @@
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
+        <v>4311</v>
+      </c>
+      <c r="B83" t="s">
         <v>4312</v>
-      </c>
-      <c r="B83" t="s">
-        <v>4313</v>
       </c>
       <c r="C83" t="s">
         <v>4155</v>
@@ -61177,10 +61204,10 @@
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
+        <v>4313</v>
+      </c>
+      <c r="B84" t="s">
         <v>4314</v>
-      </c>
-      <c r="B84" t="s">
-        <v>4315</v>
       </c>
       <c r="C84" t="s">
         <v>4155</v>
@@ -61188,10 +61215,10 @@
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
+        <v>4315</v>
+      </c>
+      <c r="B85" t="s">
         <v>4316</v>
-      </c>
-      <c r="B85" t="s">
-        <v>4317</v>
       </c>
       <c r="C85" t="s">
         <v>4155</v>
@@ -61199,10 +61226,10 @@
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
+        <v>4317</v>
+      </c>
+      <c r="B86" t="s">
         <v>4318</v>
-      </c>
-      <c r="B86" t="s">
-        <v>4319</v>
       </c>
       <c r="C86" t="s">
         <v>4155</v>
@@ -61210,10 +61237,10 @@
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
+        <v>4319</v>
+      </c>
+      <c r="B87" t="s">
         <v>4320</v>
-      </c>
-      <c r="B87" t="s">
-        <v>4321</v>
       </c>
       <c r="C87" t="s">
         <v>4155</v>
@@ -61221,21 +61248,21 @@
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
+        <v>4321</v>
+      </c>
+      <c r="B88" t="s">
         <v>4322</v>
       </c>
-      <c r="B88" t="s">
-        <v>4323</v>
-      </c>
       <c r="C88" t="s">
-        <v>4158</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
+        <v>4323</v>
+      </c>
+      <c r="B89" t="s">
         <v>4324</v>
-      </c>
-      <c r="B89" t="s">
-        <v>4325</v>
       </c>
       <c r="C89" t="s">
         <v>4155</v>
@@ -61243,21 +61270,21 @@
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
+        <v>4325</v>
+      </c>
+      <c r="B90" t="s">
         <v>4326</v>
       </c>
-      <c r="B90" t="s">
-        <v>4327</v>
-      </c>
       <c r="C90" t="s">
-        <v>4155</v>
+        <v>4158</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
+        <v>4327</v>
+      </c>
+      <c r="B91" t="s">
         <v>4328</v>
-      </c>
-      <c r="B91" t="s">
-        <v>4329</v>
       </c>
       <c r="C91" t="s">
         <v>4155</v>
@@ -61265,10 +61292,10 @@
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
+        <v>4329</v>
+      </c>
+      <c r="B92" t="s">
         <v>4330</v>
-      </c>
-      <c r="B92" t="s">
-        <v>4331</v>
       </c>
       <c r="C92" t="s">
         <v>4155</v>
@@ -61276,10 +61303,10 @@
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
+        <v>4331</v>
+      </c>
+      <c r="B93" t="s">
         <v>4332</v>
-      </c>
-      <c r="B93" t="s">
-        <v>4333</v>
       </c>
       <c r="C93" t="s">
         <v>4155</v>
@@ -61287,10 +61314,10 @@
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
+        <v>4333</v>
+      </c>
+      <c r="B94" t="s">
         <v>4334</v>
-      </c>
-      <c r="B94" t="s">
-        <v>4335</v>
       </c>
       <c r="C94" t="s">
         <v>4155</v>
@@ -61298,10 +61325,10 @@
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
+        <v>4335</v>
+      </c>
+      <c r="B95" t="s">
         <v>4336</v>
-      </c>
-      <c r="B95" t="s">
-        <v>4337</v>
       </c>
       <c r="C95" t="s">
         <v>4155</v>
@@ -61309,10 +61336,10 @@
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
+        <v>4337</v>
+      </c>
+      <c r="B96" t="s">
         <v>4338</v>
-      </c>
-      <c r="B96" t="s">
-        <v>4339</v>
       </c>
       <c r="C96" t="s">
         <v>4155</v>
@@ -61320,13 +61347,13 @@
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
+        <v>4339</v>
+      </c>
+      <c r="B97" t="s">
         <v>4340</v>
       </c>
-      <c r="B97" t="s">
-        <v>4177</v>
-      </c>
       <c r="C97" t="s">
-        <v>4163</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -61345,29 +61372,29 @@
         <v>4343</v>
       </c>
       <c r="B99" t="s">
-        <v>4344</v>
+        <v>4177</v>
       </c>
       <c r="C99" t="s">
-        <v>4155</v>
+        <v>4163</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
+        <v>4344</v>
+      </c>
+      <c r="B100" t="s">
         <v>4345</v>
       </c>
-      <c r="B100" t="s">
-        <v>4346</v>
-      </c>
       <c r="C100" t="s">
-        <v>4158</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
+        <v>4346</v>
+      </c>
+      <c r="B101" t="s">
         <v>4347</v>
-      </c>
-      <c r="B101" t="s">
-        <v>4348</v>
       </c>
       <c r="C101" t="s">
         <v>4155</v>
@@ -61375,10 +61402,10 @@
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
+        <v>4348</v>
+      </c>
+      <c r="B102" t="s">
         <v>4349</v>
-      </c>
-      <c r="B102" t="s">
-        <v>4350</v>
       </c>
       <c r="C102" t="s">
         <v>4155</v>
@@ -61386,24 +61413,24 @@
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
+        <v>4350</v>
+      </c>
+      <c r="B103" t="s">
         <v>4351</v>
       </c>
-      <c r="B103" t="s">
-        <v>4352</v>
-      </c>
       <c r="C103" t="s">
-        <v>4155</v>
+        <v>4158</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
+        <v>4352</v>
+      </c>
+      <c r="B104" t="s">
         <v>4353</v>
       </c>
-      <c r="B104" t="s">
-        <v>4216</v>
-      </c>
       <c r="C104" t="s">
-        <v>4158</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -61433,18 +61460,18 @@
         <v>4358</v>
       </c>
       <c r="B107" t="s">
-        <v>4359</v>
+        <v>4218</v>
       </c>
       <c r="C107" t="s">
-        <v>4155</v>
+        <v>4158</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
+        <v>4359</v>
+      </c>
+      <c r="B108" t="s">
         <v>4360</v>
-      </c>
-      <c r="B108" t="s">
-        <v>4361</v>
       </c>
       <c r="C108" t="s">
         <v>4155</v>
@@ -61452,10 +61479,10 @@
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
+        <v>4361</v>
+      </c>
+      <c r="B109" t="s">
         <v>4362</v>
-      </c>
-      <c r="B109" t="s">
-        <v>4307</v>
       </c>
       <c r="C109" t="s">
         <v>4155</v>
@@ -61488,7 +61515,7 @@
         <v>4367</v>
       </c>
       <c r="B112" t="s">
-        <v>4307</v>
+        <v>4310</v>
       </c>
       <c r="C112" t="s">
         <v>4155</v>
@@ -61499,7 +61526,7 @@
         <v>4368</v>
       </c>
       <c r="B113" t="s">
-        <v>4206</v>
+        <v>4369</v>
       </c>
       <c r="C113" t="s">
         <v>4155</v>
@@ -61507,24 +61534,24 @@
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>4369</v>
+        <v>4370</v>
       </c>
       <c r="B114" t="s">
-        <v>4370</v>
+        <v>4371</v>
       </c>
       <c r="C114" t="s">
-        <v>4163</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>4371</v>
+        <v>4372</v>
       </c>
       <c r="B115" t="s">
-        <v>4372</v>
+        <v>4310</v>
       </c>
       <c r="C115" t="s">
-        <v>4158</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -61532,7 +61559,7 @@
         <v>4373</v>
       </c>
       <c r="B116" t="s">
-        <v>4311</v>
+        <v>4206</v>
       </c>
       <c r="C116" t="s">
         <v>4155</v>
@@ -61543,29 +61570,29 @@
         <v>4374</v>
       </c>
       <c r="B117" t="s">
-        <v>4233</v>
+        <v>4375</v>
       </c>
       <c r="C117" t="s">
-        <v>4155</v>
+        <v>4163</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>4375</v>
+        <v>4376</v>
       </c>
       <c r="B118" t="s">
-        <v>4376</v>
+        <v>4377</v>
       </c>
       <c r="C118" t="s">
-        <v>4155</v>
+        <v>4158</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>4377</v>
+        <v>4378</v>
       </c>
       <c r="B119" t="s">
-        <v>4378</v>
+        <v>4314</v>
       </c>
       <c r="C119" t="s">
         <v>4155</v>
@@ -61576,7 +61603,7 @@
         <v>4379</v>
       </c>
       <c r="B120" t="s">
-        <v>4380</v>
+        <v>4235</v>
       </c>
       <c r="C120" t="s">
         <v>4155</v>
@@ -61584,21 +61611,21 @@
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
+        <v>4380</v>
+      </c>
+      <c r="B121" t="s">
         <v>4381</v>
       </c>
-      <c r="B121" t="s">
-        <v>4382</v>
-      </c>
       <c r="C121" t="s">
-        <v>4158</v>
+        <v>4155</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
+        <v>4382</v>
+      </c>
+      <c r="B122" t="s">
         <v>4383</v>
-      </c>
-      <c r="B122" t="s">
-        <v>4384</v>
       </c>
       <c r="C122" t="s">
         <v>4155</v>
@@ -61606,12 +61633,67 @@
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
+        <v>4384</v>
+      </c>
+      <c r="B123" t="s">
         <v>4385</v>
       </c>
-      <c r="B123" t="s">
+      <c r="C123" t="s">
+        <v>4155</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3">
+      <c r="A124" t="s">
         <v>4386</v>
       </c>
-      <c r="C123" t="s">
+      <c r="B124" t="s">
+        <v>4387</v>
+      </c>
+      <c r="C124" t="s">
+        <v>4155</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3">
+      <c r="A125" t="s">
+        <v>4388</v>
+      </c>
+      <c r="B125" t="s">
+        <v>4389</v>
+      </c>
+      <c r="C125" t="s">
+        <v>4155</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3">
+      <c r="A126" t="s">
+        <v>4390</v>
+      </c>
+      <c r="B126" t="s">
+        <v>4391</v>
+      </c>
+      <c r="C126" t="s">
+        <v>4158</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3">
+      <c r="A127" t="s">
+        <v>4392</v>
+      </c>
+      <c r="B127" t="s">
+        <v>4393</v>
+      </c>
+      <c r="C127" t="s">
+        <v>4155</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3">
+      <c r="A128" t="s">
+        <v>4394</v>
+      </c>
+      <c r="B128" t="s">
+        <v>4395</v>
+      </c>
+      <c r="C128" t="s">
         <v>4155</v>
       </c>
     </row>

</xml_diff>